<commit_message>
fix: HĐ Truc Vien 103 bỏ nệm, HĐ 201 Diệu thêm CCCD
</commit_message>
<xml_diff>
--- a/TT/TT_CCCD.xlsx
+++ b/TT/TT_CCCD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tro\TT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB8D40D8-A0F5-4F07-AC63-6D8F7435D2DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B3D69D8-7B0D-4286-8DBE-BE0153D3AB40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6000" yWindow="3570" windowWidth="18000" windowHeight="9210" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1008,6 +1008,11 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="A14:A16"/>
     <mergeCell ref="A32:A34"/>
     <mergeCell ref="A35:A37"/>
     <mergeCell ref="A38:A40"/>
@@ -1017,11 +1022,6 @@
     <mergeCell ref="A23:A25"/>
     <mergeCell ref="A26:A28"/>
     <mergeCell ref="A29:A31"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="A14:A16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>